<commit_message>
formatos cambiados listo para subir a produccion
</commit_message>
<xml_diff>
--- a/public/report_templates/caja/reportes/vchAdelanto.xlsx
+++ b/public/report_templates/caja/reportes/vchAdelanto.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\CredypymeApp\public\report_templates\caja\reportes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\CredypymeApp\public\report_templates\caja\reportes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C18C00-4E25-4DD4-9CAE-DDD60A133F82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D7A2A6-1499-4467-8D82-ABA7DBA4BB31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AFC928B-410F-4A53-A090-F50511B27738}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{9AFC928B-410F-4A53-A090-F50511B27738}"/>
   </bookViews>
   <sheets>
     <sheet name="vchDesembolso" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>(concepto)</t>
   </si>
@@ -71,7 +71,10 @@
     <t>(titulo)</t>
   </si>
   <si>
-    <t>CREDIPYME HUANCA SAC</t>
+    <t>CREDIPYME HUANCA S.A.C</t>
+  </si>
+  <si>
+    <t>RUC: 20614827239</t>
   </si>
 </sst>
 </file>
@@ -190,25 +193,25 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="22" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -542,16 +545,18 @@
       <c r="C1" s="7"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
+      <c r="A2" s="7" t="s">
+        <v>13</v>
+      </c>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
     </row>
     <row r="4" spans="1:5" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -568,18 +573,18 @@
       <c r="C5" s="9"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -591,18 +596,18 @@
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="10"/>
+      <c r="B10" s="6"/>
       <c r="C10" s="5" t="s">
         <v>6</v>
       </c>
@@ -620,11 +625,11 @@
       <c r="C12" s="7"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
@@ -635,6 +640,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="A7:C7"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A13:C13"/>
@@ -642,11 +652,6 @@
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="B5:C5"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.27559055118110237" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>